<commit_message>
move file out to test action
</commit_message>
<xml_diff>
--- a/data/boprc_cyano/og_excel_files/Cyanobacteria Report-20250306 (1).xlsx
+++ b/data/boprc_cyano/og_excel_files/Cyanobacteria Report-20250306 (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnnaR\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://waikatouniversitynz-my.sharepoint.com/personal/whitney_woelmer_waikato_ac_nz/Documents/Desktop/lakecast_rotorua/data/boprc_cyano/og_excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41FE1868-D7EB-467F-93FB-187FF8D6ABE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{41FE1868-D7EB-467F-93FB-187FF8D6ABE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AA40618-B717-41CA-B7F4-9E8C1A89FBE7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="86280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lakes Data" sheetId="2" r:id="rId1"/>
@@ -20,9 +20,9 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="52" r:id="rId5"/>
-    <pivotCache cacheId="59" r:id="rId6"/>
-    <pivotCache cacheId="65" r:id="rId7"/>
+    <pivotCache cacheId="30" r:id="rId5"/>
+    <pivotCache cacheId="37" r:id="rId6"/>
+    <pivotCache cacheId="43" r:id="rId7"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -619,16 +619,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,7 +648,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Anna Raeburn" refreshedDate="45722.642029629627" refreshedVersion="8" recordCount="96" xr:uid="{00000000-000A-0000-FFFF-FFFF02000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="45989.421394675926" refreshedVersion="8" recordCount="96" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P97" sheet="Lakes Data"/>
   </cacheSource>
@@ -732,7 +733,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Anna Raeburn" refreshedDate="45722.642029745373" refreshedVersion="8" recordCount="22" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="45989.421394791665" refreshedVersion="8" recordCount="22" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P23" sheet="Toxin Data"/>
   </cacheSource>
@@ -818,7 +819,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Anna Raeburn" refreshedDate="45722.642030092589" refreshedVersion="8" recordCount="96" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="45989.421394907411" refreshedVersion="8" recordCount="96" xr:uid="{00000000-000A-0000-FFFF-FFFF02000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P97" sheet="Lakes Data"/>
   </cacheSource>
@@ -4770,7 +4771,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000000000000}" name="AlertWarning" cacheId="65" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000000000000}" name="AlertWarning" cacheId="30" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
   <location ref="A8:D23" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
   <pivotFields count="16">
     <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
@@ -4895,126 +4896,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000002000000}" name="AlertWarning" cacheId="52" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
-  <location ref="A37:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
-  <pivotFields count="16">
-    <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Location" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField name="Site" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="13">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-      </items>
-    </pivotField>
-    <pivotField name="Dates" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="1">
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField name="MicroscopeType" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="WholePlate" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Species" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="IsSpeciesToxic" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="VolumeInMillilitres" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Average" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="NumberOfColonies" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="CellsPerMl" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="TotalBioVolume" dataField="1" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="PotentiallyToxicCellMl" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="PotentiallyToxicBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="ToxinCluster" compact="0" outline="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="1"/>
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="13">
-    <i>
-      <x/>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="3"/>
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="4"/>
-      <x v="5"/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="3"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="TotalBioVolume" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000001000000}" name="CellsPermL" cacheId="59" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000001000000}" name="CellsPermL" cacheId="37" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
   <location ref="A8:D22" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
   <pivotFields count="16">
     <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
@@ -5123,6 +5005,125 @@
   </colItems>
   <dataFields count="1">
     <dataField name="CellsPerMl" fld="11" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000002000000}" name="AlertWarning" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+  <location ref="A37:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
+  <pivotFields count="16">
+    <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Location" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+      </items>
+    </pivotField>
+    <pivotField name="Site" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="13">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+      </items>
+    </pivotField>
+    <pivotField name="Dates" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField name="MicroscopeType" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="WholePlate" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Species" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="IsSpeciesToxic" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="VolumeInMillilitres" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Average" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="NumberOfColonies" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="CellsPerMl" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="TotalBioVolume" dataField="1" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="PotentiallyToxicCellMl" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="PotentiallyToxicBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="ToxinCluster" compact="0" outline="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="13">
+    <i>
+      <x/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="3"/>
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="4"/>
+      <x v="5"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="3"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="TotalBioVolume" fld="12" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
   <extLst>
@@ -5469,27 +5470,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P97"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
-    <col min="7" max="7" width="32.140625" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" customWidth="1"/>
-    <col min="11" max="11" width="20.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" customWidth="1"/>
-    <col min="13" max="13" width="22.5703125" customWidth="1"/>
-    <col min="14" max="14" width="23.42578125" customWidth="1"/>
-    <col min="15" max="15" width="27.42578125" customWidth="1"/>
-    <col min="16" max="16" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="12.41796875" customWidth="1"/>
+    <col min="2" max="2" width="11.83984375" customWidth="1"/>
+    <col min="3" max="3" width="13.83984375" customWidth="1"/>
+    <col min="4" max="4" width="14.83984375" customWidth="1"/>
+    <col min="5" max="5" width="18.578125" customWidth="1"/>
+    <col min="6" max="6" width="14.41796875" customWidth="1"/>
+    <col min="7" max="7" width="32.15625" customWidth="1"/>
+    <col min="8" max="8" width="16.578125" customWidth="1"/>
+    <col min="9" max="9" width="20.68359375" customWidth="1"/>
+    <col min="10" max="10" width="18.26171875" customWidth="1"/>
+    <col min="11" max="11" width="20.83984375" customWidth="1"/>
+    <col min="12" max="12" width="18.26171875" customWidth="1"/>
+    <col min="13" max="13" width="22.578125" customWidth="1"/>
+    <col min="14" max="14" width="23.41796875" customWidth="1"/>
+    <col min="15" max="15" width="27.41796875" customWidth="1"/>
+    <col min="16" max="16" width="15.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5539,7 +5540,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -5583,7 +5584,7 @@
         <v>0.187647602083334</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -5630,7 +5631,7 @@
         <v>0.27705588822916599</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -5674,7 +5675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -5721,7 +5722,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -5765,7 +5766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -5812,7 +5813,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -5856,7 +5857,7 @@
         <v>1.975E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -5903,7 +5904,7 @@
         <v>0.1090463634</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>41</v>
       </c>
@@ -5947,7 +5948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -5991,7 +5992,7 @@
         <v>5.13E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -6035,7 +6036,7 @@
         <v>1.7160000000000001E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -6082,7 +6083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -6132,7 +6133,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -6176,7 +6177,7 @@
         <v>9.2678039999999993E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -6220,7 +6221,7 @@
         <v>1.8810000000000001E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -6267,7 +6268,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -6311,7 +6312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>56</v>
       </c>
@@ -6355,7 +6356,7 @@
         <v>6.0039999999999996E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>57</v>
       </c>
@@ -6399,7 +6400,7 @@
         <v>3.0339999999999998E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -6446,7 +6447,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -6490,7 +6491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -6534,7 +6535,7 @@
         <v>7.6538799999999998E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -6578,7 +6579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -6628,7 +6629,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -6672,7 +6673,7 @@
         <v>1.17294673888889E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -6719,7 +6720,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
         <v>69</v>
       </c>
@@ -6763,7 +6764,7 @@
         <v>3.5814208333333299E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -6810,7 +6811,7 @@
         <v>4.9494900000000001E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
         <v>73</v>
       </c>
@@ -6854,7 +6855,7 @@
         <v>5.0253371999999998E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -6901,7 +6902,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
         <v>75</v>
       </c>
@@ -6948,7 +6949,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -6992,7 +6993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
         <v>77</v>
       </c>
@@ -7036,7 +7037,7 @@
         <v>9.1E-4</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
         <v>78</v>
       </c>
@@ -7080,7 +7081,7 @@
         <v>2.0540000000000001E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
         <v>79</v>
       </c>
@@ -7124,7 +7125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
         <v>82</v>
       </c>
@@ -7174,7 +7175,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
         <v>83</v>
       </c>
@@ -7218,7 +7219,7 @@
         <v>2.1459999999999999E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>84</v>
       </c>
@@ -7262,7 +7263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
         <v>85</v>
       </c>
@@ -7309,7 +7310,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
         <v>86</v>
       </c>
@@ -7353,7 +7354,7 @@
         <v>1.027E-4</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
         <v>87</v>
       </c>
@@ -7397,7 +7398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>88</v>
       </c>
@@ -7441,7 +7442,7 @@
         <v>5.9400000000000002E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>89</v>
       </c>
@@ -7485,7 +7486,7 @@
         <v>3.2235839999999998E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>90</v>
       </c>
@@ -7529,7 +7530,7 @@
         <v>8.7739600000000001E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -7573,7 +7574,7 @@
         <v>5.3200000000000003E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
         <v>92</v>
       </c>
@@ -7623,7 +7624,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -7667,7 +7668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
         <v>95</v>
       </c>
@@ -7711,7 +7712,7 @@
         <v>9.7295265972222197E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
         <v>96</v>
       </c>
@@ -7755,7 +7756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>98</v>
       </c>
@@ -7799,7 +7800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
         <v>99</v>
       </c>
@@ -7843,7 +7844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
         <v>101</v>
       </c>
@@ -7887,7 +7888,7 @@
         <v>3.1083088580555598E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" t="s">
         <v>102</v>
       </c>
@@ -7937,7 +7938,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" t="s">
         <v>104</v>
       </c>
@@ -7984,7 +7985,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" t="s">
         <v>105</v>
       </c>
@@ -8028,7 +8029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" t="s">
         <v>106</v>
       </c>
@@ -8072,7 +8073,7 @@
         <v>1.325428E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" t="s">
         <v>107</v>
       </c>
@@ -8116,7 +8117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" t="s">
         <v>108</v>
       </c>
@@ -8160,7 +8161,7 @@
         <v>2.244996E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" t="s">
         <v>109</v>
       </c>
@@ -8204,7 +8205,7 @@
         <v>5.9400000000000002E-4</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" t="s">
         <v>110</v>
       </c>
@@ -8248,7 +8249,7 @@
         <v>1.6798E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" t="s">
         <v>111</v>
       </c>
@@ -8292,7 +8293,7 @@
         <v>4.75E-4</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" t="s">
         <v>112</v>
       </c>
@@ -8336,7 +8337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" t="s">
         <v>113</v>
       </c>
@@ -8380,7 +8381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" t="s">
         <v>115</v>
       </c>
@@ -8424,7 +8425,7 @@
         <v>7.2000000000000002E-5</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" t="s">
         <v>117</v>
       </c>
@@ -8468,7 +8469,7 @@
         <v>6.3200000000000005E-5</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" t="s">
         <v>118</v>
       </c>
@@ -8512,7 +8513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" t="s">
         <v>120</v>
       </c>
@@ -8556,7 +8557,7 @@
         <v>5.1145202777777898E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" t="s">
         <v>121</v>
       </c>
@@ -8603,7 +8604,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" t="s">
         <v>122</v>
       </c>
@@ -8647,7 +8648,7 @@
         <v>3.7667750694444398E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" t="s">
         <v>123</v>
       </c>
@@ -8691,7 +8692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" t="s">
         <v>124</v>
       </c>
@@ -8735,7 +8736,7 @@
         <v>2.4818618055555499E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" t="s">
         <v>125</v>
       </c>
@@ -8782,7 +8783,7 @@
         <v>4.2735000000000002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" t="s">
         <v>127</v>
       </c>
@@ -8832,7 +8833,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" t="s">
         <v>128</v>
       </c>
@@ -8876,7 +8877,7 @@
         <v>8.4043439999999994E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" t="s">
         <v>129</v>
       </c>
@@ -8923,7 +8924,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" t="s">
         <v>130</v>
       </c>
@@ -8967,7 +8968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" t="s">
         <v>131</v>
       </c>
@@ -9014,7 +9015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" t="s">
         <v>133</v>
       </c>
@@ -9064,7 +9065,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" t="s">
         <v>134</v>
       </c>
@@ -9108,7 +9109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" t="s">
         <v>135</v>
       </c>
@@ -9152,7 +9153,7 @@
         <v>1.5312024E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" t="s">
         <v>136</v>
       </c>
@@ -9196,7 +9197,7 @@
         <v>4.2180000000000004E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" t="s">
         <v>137</v>
       </c>
@@ -9243,7 +9244,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" t="s">
         <v>138</v>
       </c>
@@ -9287,7 +9288,7 @@
         <v>5.7200000000000003E-4</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" t="s">
         <v>139</v>
       </c>
@@ -9331,7 +9332,7 @@
         <v>1.896E-4</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" t="s">
         <v>140</v>
       </c>
@@ -9375,7 +9376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" t="s">
         <v>141</v>
       </c>
@@ -9419,7 +9420,7 @@
         <v>1.887E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" t="s">
         <v>143</v>
       </c>
@@ -9466,7 +9467,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" t="s">
         <v>144</v>
       </c>
@@ -9513,7 +9514,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" t="s">
         <v>145</v>
       </c>
@@ -9557,7 +9558,7 @@
         <v>2.5280000000000002E-4</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" t="s">
         <v>146</v>
       </c>
@@ -9601,7 +9602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" t="s">
         <v>147</v>
       </c>
@@ -9645,7 +9646,7 @@
         <v>2.935764E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A93" t="s">
         <v>148</v>
       </c>
@@ -9689,7 +9690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" t="s">
         <v>149</v>
       </c>
@@ -9733,7 +9734,7 @@
         <v>2.1882999999999998E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" t="s">
         <v>151</v>
       </c>
@@ -9777,7 +9778,7 @@
         <v>8.0589599999999996E-4</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" t="s">
         <v>152</v>
       </c>
@@ -9821,7 +9822,7 @@
         <v>2.0349999999999999E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" t="s">
         <v>153</v>
       </c>
@@ -9879,27 +9880,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
-    <col min="7" max="7" width="22.28515625" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" customWidth="1"/>
-    <col min="11" max="11" width="20.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" customWidth="1"/>
-    <col min="14" max="14" width="23.42578125" customWidth="1"/>
-    <col min="15" max="15" width="27.42578125" customWidth="1"/>
-    <col min="16" max="16" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="12.41796875" customWidth="1"/>
+    <col min="2" max="2" width="11.83984375" customWidth="1"/>
+    <col min="3" max="3" width="13.83984375" customWidth="1"/>
+    <col min="4" max="4" width="14.83984375" customWidth="1"/>
+    <col min="5" max="5" width="18.578125" customWidth="1"/>
+    <col min="6" max="6" width="14.41796875" customWidth="1"/>
+    <col min="7" max="7" width="22.26171875" customWidth="1"/>
+    <col min="8" max="8" width="16.578125" customWidth="1"/>
+    <col min="9" max="9" width="20.68359375" customWidth="1"/>
+    <col min="10" max="10" width="18.26171875" customWidth="1"/>
+    <col min="11" max="11" width="20.83984375" customWidth="1"/>
+    <col min="12" max="12" width="18.26171875" customWidth="1"/>
+    <col min="13" max="13" width="20.41796875" customWidth="1"/>
+    <col min="14" max="14" width="23.41796875" customWidth="1"/>
+    <col min="15" max="15" width="27.41796875" customWidth="1"/>
+    <col min="16" max="16" width="15.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9949,7 +9950,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -9996,7 +9997,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -10043,7 +10044,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>50</v>
       </c>
@@ -10093,7 +10094,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -10140,7 +10141,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>58</v>
       </c>
@@ -10187,7 +10188,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -10237,7 +10238,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>68</v>
       </c>
@@ -10284,7 +10285,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>74</v>
       </c>
@@ -10331,7 +10332,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>75</v>
       </c>
@@ -10378,7 +10379,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>82</v>
       </c>
@@ -10428,7 +10429,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -10475,7 +10476,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>92</v>
       </c>
@@ -10525,7 +10526,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>102</v>
       </c>
@@ -10575,7 +10576,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>104</v>
       </c>
@@ -10622,7 +10623,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>121</v>
       </c>
@@ -10669,7 +10670,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>127</v>
       </c>
@@ -10719,7 +10720,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>129</v>
       </c>
@@ -10766,7 +10767,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>133</v>
       </c>
@@ -10816,7 +10817,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>137</v>
       </c>
@@ -10863,7 +10864,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>143</v>
       </c>
@@ -10910,7 +10911,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>144</v>
       </c>
@@ -10957,7 +10958,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>153</v>
       </c>
@@ -11015,13 +11016,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="32.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>154</v>
       </c>
@@ -11029,7 +11030,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>156</v>
       </c>
@@ -11037,7 +11038,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>157</v>
       </c>
@@ -11045,7 +11046,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>159</v>
       </c>
@@ -11053,7 +11054,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C8" s="6" t="s">
         <v>174</v>
       </c>
@@ -11061,12 +11062,12 @@
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="6" t="s">
         <v>1</v>
       </c>
@@ -11080,161 +11081,161 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="7">
         <v>0.72984618604355433</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="7">
         <v>0.71855842722411012</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" t="s">
         <v>48</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="7">
         <v>4.7560744483191204E-2</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="7">
         <v>4.6962224483191199E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>103</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>6.1660725999999999E-2</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="7">
         <v>6.069119600000001E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" t="s">
         <v>119</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="7">
         <v>0.1087837414361211</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="7">
         <v>0.10866310410278775</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" t="s">
         <v>132</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>3.1795496299443803E-2</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="7">
         <v>3.1440886299443804E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>35</v>
       </c>
       <c r="B16" t="s">
         <v>36</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="7">
         <v>0.11608986339999999</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="7">
         <v>0.11608986339999999</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>65</v>
       </c>
       <c r="B17" t="s">
         <v>66</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="7">
         <v>0.36331107890694442</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="7">
         <v>0.36331107890694442</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" t="s">
         <v>93</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="7">
         <v>0.3330695613902781</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="7">
         <v>0.32735455621944476</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>71</v>
       </c>
       <c r="B19" t="s">
         <v>72</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="7">
         <v>0.12800909114220399</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="7">
         <v>0.127194891142204</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B20" t="s">
         <v>126</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="7">
         <v>7.5128383920372105E-2</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="7">
         <v>7.4815583920372103E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" t="s">
         <v>142</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="7">
         <v>1.9412851571276001E-2</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="7">
         <v>1.9315051571276002E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B22" t="s">
         <v>150</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="7">
         <v>5.1153542857039994E-3</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="7">
         <v>5.1153542857039994E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>80</v>
       </c>
       <c r="B23" t="s">
         <v>81</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="7">
         <v>3.0247895141226E-2</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="7">
         <v>2.9875095141226E-2</v>
       </c>
     </row>
@@ -11246,15 +11247,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" customWidth="1"/>
-    <col min="2" max="2" width="33.7109375" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="29.5703125" customWidth="1"/>
+    <col min="1" max="1" width="24.578125" customWidth="1"/>
+    <col min="2" max="2" width="33.68359375" customWidth="1"/>
+    <col min="3" max="3" width="31.41796875" customWidth="1"/>
+    <col min="4" max="4" width="29.578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>161</v>
       </c>
@@ -11268,7 +11269,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>165</v>
       </c>
@@ -11282,7 +11283,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>166</v>
       </c>
@@ -11296,7 +11297,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>170</v>
       </c>
@@ -11310,7 +11311,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
@@ -11321,12 +11322,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="6" t="s">
         <v>1</v>
       </c>
@@ -11337,135 +11338,135 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="7">
         <v>2472.4370138888848</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" t="s">
         <v>48</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="7">
         <v>378.66</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>103</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>368.4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" t="s">
         <v>119</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="7">
         <v>241.90298611111101</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" t="s">
         <v>132</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>98.990000000000009</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>65</v>
       </c>
       <c r="B16" t="s">
         <v>66</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="7">
         <v>3669.8567951388891</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B17" t="s">
         <v>93</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="7">
         <v>2287.0827777777799</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>71</v>
       </c>
       <c r="B18" t="s">
         <v>72</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="7">
         <v>185.8</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" t="s">
         <v>126</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="7">
         <v>201.155</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B20" t="s">
         <v>142</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="7">
         <v>85.899999999999991</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" t="s">
         <v>150</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="7">
         <v>1.2</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>80</v>
       </c>
       <c r="B22" t="s">
         <v>81</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="7">
         <v>236.20000000000002</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="3" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="4" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="6" t="s">
         <v>12</v>
       </c>
@@ -11473,7 +11474,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="6" t="s">
         <v>1</v>
       </c>
@@ -11484,122 +11485,122 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>17</v>
       </c>
       <c r="B39" t="s">
         <v>18</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="7">
         <v>0.72984618604355433</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B40" t="s">
         <v>48</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="7">
         <v>4.7560744483191204E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B41" t="s">
         <v>103</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="7">
         <v>6.1660725999999999E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B42" t="s">
         <v>119</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="7">
         <v>0.1087837414361211</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B43" t="s">
         <v>132</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="7">
         <v>3.1795496299443803E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>35</v>
       </c>
       <c r="B44" t="s">
         <v>36</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="7">
         <v>0.11608986339999999</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>65</v>
       </c>
       <c r="B45" t="s">
         <v>66</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="7">
         <v>0.36331107890694442</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B46" t="s">
         <v>93</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="7">
         <v>0.3330695613902781</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
         <v>71</v>
       </c>
       <c r="B47" t="s">
         <v>72</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="7">
         <v>0.12800909114220399</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B48" t="s">
         <v>126</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="7">
         <v>7.5128383920372105E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B49" t="s">
         <v>142</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="7">
         <v>1.9412851571276001E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B50" t="s">
         <v>150</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="7">
         <v>5.1153542857039994E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>80</v>
       </c>
       <c r="B51" t="s">
         <v>81</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="7">
         <v>3.0247895141226E-2</v>
       </c>
     </row>

</xml_diff>